<commit_message>
Done audio evaluation data collection
</commit_message>
<xml_diff>
--- a/eval/speech/recording_tracker_UPDATED.xlsx
+++ b/eval/speech/recording_tracker_UPDATED.xlsx
@@ -1,25 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2">
-  <fileVersion appName="Calc" lowestEdited="4"/>
-  <workbookPr backupFile="false" showObjects="all" date1904="false"/>
-  <workbookProtection/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Lenovo\Desktop\Natural Language Processing\NLP-BorakBot\eval\speech\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0BC4407-D4CD-4941-94B3-B9DEBD079C19}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView showHorizontalScroll="true" showVerticalScroll="true" showSheetTabs="true" xWindow="0" yWindow="0" windowWidth="16384" windowHeight="8192" tabRatio="500" firstSheet="0" activeTab="0"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="Reference" sheetId="1" state="visible" r:id="rId3"/>
-    <sheet name="Yong Vay" sheetId="2" state="visible" r:id="rId4"/>
-    <sheet name="Pei Qi" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Phase 2 (reserve)" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Reference" sheetId="1" r:id="rId1"/>
+    <sheet name="Yong Vay" sheetId="2" r:id="rId2"/>
+    <sheet name="Pei Qi" sheetId="3" r:id="rId3"/>
+    <sheet name="Phase 2 (reserve)" sheetId="4" r:id="rId4"/>
   </sheets>
   <definedNames>
-    <definedName function="false" hidden="true" localSheetId="2" name="_xlnm._FilterDatabase" vbProcedure="false">'Pei Qi'!$A$6:$H$30</definedName>
-    <definedName function="false" hidden="true" localSheetId="3" name="_xlnm._FilterDatabase" vbProcedure="false">'Phase 2 (reserve)'!$A$6:$H$54</definedName>
-    <definedName function="false" hidden="true" localSheetId="1" name="_xlnm._FilterDatabase" vbProcedure="false">'Yong Vay'!$A$6:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Pei Qi'!$A$6:$H$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Phase 2 (reserve)'!$A$6:$H$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Yong Vay'!$A$6:$H$30</definedName>
   </definedNames>
-  <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
+  <calcPr calcId="191029" iterateDelta="1E-4"/>
   <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
       <loext:extCalcPr stringRefSyntax="ExcelA1"/>
     </ext>
@@ -28,889 +42,889 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="566" uniqueCount="291">
-  <si>
-    <t xml:space="preserve">BorakBot — speech test set</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Numbers</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Say numbers EXACTLY as spelled in the reference. 4 numeric sentences use Malay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">numerals and 4 use English -- deliberate, so numeral language becomes a measured</t>
-  </si>
-  <si>
-    <t xml:space="preserve">variable. Writing RM45.90 but saying 'empat puluh lima ringgit' would score a perfect</t>
-  </si>
-  <si>
-    <t xml:space="preserve">transcription as ~8 errors, which is why references are written as spoken.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Format</t>
-  </si>
-  <si>
-    <t xml:space="preserve">16 kHz mono WAV. Record in manifest order, then:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">python scripts/prepare_audio.py --speaker yv --raw "...\my_raw"</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Design</t>
-  </si>
-  <si>
-    <t xml:space="preserve">48 sentences x 6 categories. Phase 1 = 24 each, split WITHIN each category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">(4 per speaker per category) so switch_type is never confounded with speaker.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Category</t>
-  </si>
-  <si>
-    <t xml:space="preserve">What it tests</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ms_dom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malay matrix sentence, English word inserted</t>
-  </si>
-  <si>
-    <t xml:space="preserve">en_dom</t>
-  </si>
-  <si>
-    <t xml:space="preserve">English matrix sentence, Malay discourse particles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">balanced</t>
-  </si>
-  <si>
-    <t xml:space="preserve">True intra-sentential code-switching</t>
-  </si>
-  <si>
-    <t xml:space="preserve">particles</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Discourse particles: lah / lor / meh / kan / kot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">numeric</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prices, percentages, dates -- both numeral languages</t>
-  </si>
-  <si>
-    <t xml:space="preserve">entity</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malaysian named entities: MyJPJ, KWSP, LHDN, TNB</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Prediction</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Proposal S5.6: Whisper commits to one language per segment, so 'balanced'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">and 'particles' should score worst. Confirming that is the finding.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Git</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Commit manifest.csv and results.csv. Never commit audio/ -- keep it in Drive.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recording list — Yong Vay</t>
-  </si>
-  <si>
-    <t xml:space="preserve">24 utterances, phase 1. Normal pace, quiet room, do not over-enunciate.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Read the "reference" column EXACTLY as written -- numbers are spelled out on purpose.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fill only the yellow columns. Record in this order -- prepare_audio.py pairs by position.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">reference</t>
-  </si>
-  <si>
-    <t xml:space="preserve">switch_type</t>
-  </si>
-  <si>
-    <t xml:space="preserve">numeral_lang</t>
-  </si>
-  <si>
-    <t xml:space="preserve">phase</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio_path</t>
-  </si>
-  <si>
-    <t xml:space="preserve">recorded</t>
-  </si>
-  <si>
-    <t xml:space="preserve">notes</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s01_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">macam mana nak apply lesen memandu baru</t>
-  </si>
-  <si>
-    <t xml:space="preserve">1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s01_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s02_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saya nak tanya pasal insurance kereta ni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s02_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s03_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boleh tak awak explain apa itu inflation</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s03_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s04_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nak cari tempat makan yang murah dekat sini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s04_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s09_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">how do i check my epf balance ah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s09_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s10_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">can you explain what is compound interest lah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s10_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s11_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">where can i find cheap flight ticket meh</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s11_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s12_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">i want to know how to save money properly one</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s12_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s17_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saya dah submit application tapi belum dapat approval lagi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s17_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s18_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nak tanya pasal tax relief untuk medical expenses</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s18_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s19_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">macam mana nak cancel subscription yang auto renew tu</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s19_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s20_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boleh tak explain difference antara savings dengan current account</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s20_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s25_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eh betul ke ni macam tak kena je lor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s25_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s26_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">aiyo susah sangat lah macam ni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s26_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s27_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">can one lah don't worry so much</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s27_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s28_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">wah mahal gila meh ada yang murah tak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s28_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s33_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">harga dia empat puluh lima ringgit sembilan puluh sen termasuk cukai ke tak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">malay numerals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s33_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s34_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">gaji minimum sekarang seribu lima ratus ringgit ke ah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s34_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s35_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saya nak transfer one thousand five hundred ringgit boleh tak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">english numerals</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s35_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s36_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">deadline dia thirty one august twenty twenty six kan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s36_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s41_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">macam mana nak renew roadtax kat MyJPJ</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s41_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s42_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boleh guna Touch n Go eWallet tak kat sini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s42_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s43_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saya nak semak baki KWSP guna i-Akaun</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s43_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s44_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LHDN dah buka e-Filing untuk tahun ni ke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s44_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recorded:</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recording list — Pei Qi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s05_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">camne nak transfer duit guna online banking</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s05_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s06_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saya lupa password akaun macam mana nak reset</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s06_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s07_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">berapa lama proses renew passport ambil masa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s07_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s08_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tolong bagitahu cara nak book appointment klinik</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s08_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s13_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">is it safe to invest in unit trust ke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s13_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s14_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tell me how to cook nasi lemak lah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s14_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s15_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">what time the post office close ah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s15_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s16_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">can i renew my licence online or not</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s16_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s21_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">saya nak update alamat kat identity card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s21_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s22_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">camne nak claim insurance kalau accident kereta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s22_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s23_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nak tahu requirement untuk apply credit card</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s23_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s24_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">tolong terangkan macam mana interest rate affect loan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s24_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s29_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">so how ah nak buat macam mana ni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s29_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s30_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">alamak terlupa pulak kan boleh tolong tak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s30_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s31_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ish lambat betul lah service ni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s31_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s32_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">okay lah fine saya try dulu kot</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s32_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s37_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">interest rate dia three point five percent setahun je</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s37_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s38_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kena bayar deposit dua ribu lima ratus ringgit</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s38_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s39_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">cukai jualan naik dari enam peratus ke lapan peratus ke</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s39_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s40_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">buka pukul nine in the morning tutup pukul five in the evening kan</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s40_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s45_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nak apply MyKad baru kat JPN macam mana</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s45_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s46_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">boleh bayar bil TNB guna Maybank2u tak</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s46_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s47_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Grab dengan foodpanda mana lagi murah ah</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s47_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s48_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">nak tanya pasal bantuan STR tahun ni</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s48_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Phase 2 — reserve</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Record only if a category comes out close, or for paired speaker analysis.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s01_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s01_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s02_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s02_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s03_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s03_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s04_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s04_ms_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s05_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s05_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s06_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s06_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s07_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s07_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s08_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s08_ms_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s09_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s09_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s10_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s10_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s11_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s11_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s12_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s12_en_dom_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s13_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s13_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s14_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s14_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s15_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s15_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s16_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s16_en_dom_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s17_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s17_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s18_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s18_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s19_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s19_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s20_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s20_balanced_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s21_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s21_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s22_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s22_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s23_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s23_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s24_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s24_balanced_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s25_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s25_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s26_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s26_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s27_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s27_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s28_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s28_particles_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s29_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s29_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s30_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s30_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s31_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s31_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s32_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s32_particles_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s33_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s33_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s34_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s34_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s35_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s35_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s36_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s36_numeric_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s37_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s37_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s38_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s38_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s39_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s39_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s40_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s40_numeric_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s41_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s41_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s42_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s42_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s43_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s43_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s44_pq</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s44_entity_pq.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s45_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s45_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s46_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s46_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s47_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s47_entity_yv.wav</t>
-  </si>
-  <si>
-    <t xml:space="preserve">s48_yv</t>
-  </si>
-  <si>
-    <t xml:space="preserve">audio/s48_entity_yv.wav</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="614" uniqueCount="292">
+  <si>
+    <t>BorakBot — speech test set</t>
+  </si>
+  <si>
+    <t>Numbers</t>
+  </si>
+  <si>
+    <t>Say numbers EXACTLY as spelled in the reference. 4 numeric sentences use Malay</t>
+  </si>
+  <si>
+    <t>numerals and 4 use English -- deliberate, so numeral language becomes a measured</t>
+  </si>
+  <si>
+    <t>variable. Writing RM45.90 but saying 'empat puluh lima ringgit' would score a perfect</t>
+  </si>
+  <si>
+    <t>transcription as ~8 errors, which is why references are written as spoken.</t>
+  </si>
+  <si>
+    <t>Format</t>
+  </si>
+  <si>
+    <t>16 kHz mono WAV. Record in manifest order, then:</t>
+  </si>
+  <si>
+    <t>python scripts/prepare_audio.py --speaker yv --raw "...\my_raw"</t>
+  </si>
+  <si>
+    <t>Design</t>
+  </si>
+  <si>
+    <t>48 sentences x 6 categories. Phase 1 = 24 each, split WITHIN each category</t>
+  </si>
+  <si>
+    <t>(4 per speaker per category) so switch_type is never confounded with speaker.</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>What it tests</t>
+  </si>
+  <si>
+    <t>ms_dom</t>
+  </si>
+  <si>
+    <t>Malay matrix sentence, English word inserted</t>
+  </si>
+  <si>
+    <t>en_dom</t>
+  </si>
+  <si>
+    <t>English matrix sentence, Malay discourse particles</t>
+  </si>
+  <si>
+    <t>balanced</t>
+  </si>
+  <si>
+    <t>True intra-sentential code-switching</t>
+  </si>
+  <si>
+    <t>particles</t>
+  </si>
+  <si>
+    <t>Discourse particles: lah / lor / meh / kan / kot</t>
+  </si>
+  <si>
+    <t>numeric</t>
+  </si>
+  <si>
+    <t>Prices, percentages, dates -- both numeral languages</t>
+  </si>
+  <si>
+    <t>entity</t>
+  </si>
+  <si>
+    <t>Malaysian named entities: MyJPJ, KWSP, LHDN, TNB</t>
+  </si>
+  <si>
+    <t>Prediction</t>
+  </si>
+  <si>
+    <t>Proposal S5.6: Whisper commits to one language per segment, so 'balanced'</t>
+  </si>
+  <si>
+    <t>and 'particles' should score worst. Confirming that is the finding.</t>
+  </si>
+  <si>
+    <t>Git</t>
+  </si>
+  <si>
+    <t>Commit manifest.csv and results.csv. Never commit audio/ -- keep it in Drive.</t>
+  </si>
+  <si>
+    <t>Recording list — Yong Vay</t>
+  </si>
+  <si>
+    <t>24 utterances, phase 1. Normal pace, quiet room, do not over-enunciate.</t>
+  </si>
+  <si>
+    <t>Read the "reference" column EXACTLY as written -- numbers are spelled out on purpose.</t>
+  </si>
+  <si>
+    <t>Fill only the yellow columns. Record in this order -- prepare_audio.py pairs by position.</t>
+  </si>
+  <si>
+    <t>id</t>
+  </si>
+  <si>
+    <t>reference</t>
+  </si>
+  <si>
+    <t>switch_type</t>
+  </si>
+  <si>
+    <t>numeral_lang</t>
+  </si>
+  <si>
+    <t>phase</t>
+  </si>
+  <si>
+    <t>audio_path</t>
+  </si>
+  <si>
+    <t>recorded</t>
+  </si>
+  <si>
+    <t>notes</t>
+  </si>
+  <si>
+    <t>s01_yv</t>
+  </si>
+  <si>
+    <t>macam mana nak apply lesen memandu baru</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>audio/s01_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s02_yv</t>
+  </si>
+  <si>
+    <t>saya nak tanya pasal insurance kereta ni</t>
+  </si>
+  <si>
+    <t>audio/s02_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s03_yv</t>
+  </si>
+  <si>
+    <t>boleh tak awak explain apa itu inflation</t>
+  </si>
+  <si>
+    <t>audio/s03_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s04_yv</t>
+  </si>
+  <si>
+    <t>nak cari tempat makan yang murah dekat sini</t>
+  </si>
+  <si>
+    <t>audio/s04_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s09_yv</t>
+  </si>
+  <si>
+    <t>how do i check my epf balance ah</t>
+  </si>
+  <si>
+    <t>audio/s09_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s10_yv</t>
+  </si>
+  <si>
+    <t>can you explain what is compound interest lah</t>
+  </si>
+  <si>
+    <t>audio/s10_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s11_yv</t>
+  </si>
+  <si>
+    <t>where can i find cheap flight ticket meh</t>
+  </si>
+  <si>
+    <t>audio/s11_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s12_yv</t>
+  </si>
+  <si>
+    <t>i want to know how to save money properly one</t>
+  </si>
+  <si>
+    <t>audio/s12_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s17_yv</t>
+  </si>
+  <si>
+    <t>saya dah submit application tapi belum dapat approval lagi</t>
+  </si>
+  <si>
+    <t>audio/s17_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s18_yv</t>
+  </si>
+  <si>
+    <t>nak tanya pasal tax relief untuk medical expenses</t>
+  </si>
+  <si>
+    <t>audio/s18_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s19_yv</t>
+  </si>
+  <si>
+    <t>macam mana nak cancel subscription yang auto renew tu</t>
+  </si>
+  <si>
+    <t>audio/s19_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s20_yv</t>
+  </si>
+  <si>
+    <t>boleh tak explain difference antara savings dengan current account</t>
+  </si>
+  <si>
+    <t>audio/s20_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s25_yv</t>
+  </si>
+  <si>
+    <t>eh betul ke ni macam tak kena je lor</t>
+  </si>
+  <si>
+    <t>audio/s25_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s26_yv</t>
+  </si>
+  <si>
+    <t>aiyo susah sangat lah macam ni</t>
+  </si>
+  <si>
+    <t>audio/s26_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s27_yv</t>
+  </si>
+  <si>
+    <t>can one lah don't worry so much</t>
+  </si>
+  <si>
+    <t>audio/s27_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s28_yv</t>
+  </si>
+  <si>
+    <t>wah mahal gila meh ada yang murah tak</t>
+  </si>
+  <si>
+    <t>audio/s28_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s33_yv</t>
+  </si>
+  <si>
+    <t>harga dia empat puluh lima ringgit sembilan puluh sen termasuk cukai ke tak</t>
+  </si>
+  <si>
+    <t>malay numerals</t>
+  </si>
+  <si>
+    <t>audio/s33_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s34_yv</t>
+  </si>
+  <si>
+    <t>gaji minimum sekarang seribu lima ratus ringgit ke ah</t>
+  </si>
+  <si>
+    <t>audio/s34_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s35_yv</t>
+  </si>
+  <si>
+    <t>saya nak transfer one thousand five hundred ringgit boleh tak</t>
+  </si>
+  <si>
+    <t>english numerals</t>
+  </si>
+  <si>
+    <t>audio/s35_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s36_yv</t>
+  </si>
+  <si>
+    <t>deadline dia thirty one august twenty twenty six kan</t>
+  </si>
+  <si>
+    <t>audio/s36_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s41_yv</t>
+  </si>
+  <si>
+    <t>macam mana nak renew roadtax kat MyJPJ</t>
+  </si>
+  <si>
+    <t>audio/s41_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>s42_yv</t>
+  </si>
+  <si>
+    <t>boleh guna Touch n Go eWallet tak kat sini</t>
+  </si>
+  <si>
+    <t>audio/s42_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>s43_yv</t>
+  </si>
+  <si>
+    <t>saya nak semak baki KWSP guna i-Akaun</t>
+  </si>
+  <si>
+    <t>audio/s43_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>s44_yv</t>
+  </si>
+  <si>
+    <t>LHDN dah buka e-Filing untuk tahun ni ke</t>
+  </si>
+  <si>
+    <t>audio/s44_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>Recorded:</t>
+  </si>
+  <si>
+    <t>Recording list — Pei Qi</t>
+  </si>
+  <si>
+    <t>s05_pq</t>
+  </si>
+  <si>
+    <t>camne nak transfer duit guna online banking</t>
+  </si>
+  <si>
+    <t>audio/s05_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s06_pq</t>
+  </si>
+  <si>
+    <t>saya lupa password akaun macam mana nak reset</t>
+  </si>
+  <si>
+    <t>audio/s06_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s07_pq</t>
+  </si>
+  <si>
+    <t>berapa lama proses renew passport ambil masa</t>
+  </si>
+  <si>
+    <t>audio/s07_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s08_pq</t>
+  </si>
+  <si>
+    <t>tolong bagitahu cara nak book appointment klinik</t>
+  </si>
+  <si>
+    <t>audio/s08_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s13_pq</t>
+  </si>
+  <si>
+    <t>is it safe to invest in unit trust ke</t>
+  </si>
+  <si>
+    <t>audio/s13_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s14_pq</t>
+  </si>
+  <si>
+    <t>tell me how to cook nasi lemak lah</t>
+  </si>
+  <si>
+    <t>audio/s14_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s15_pq</t>
+  </si>
+  <si>
+    <t>what time the post office close ah</t>
+  </si>
+  <si>
+    <t>audio/s15_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s16_pq</t>
+  </si>
+  <si>
+    <t>can i renew my licence online or not</t>
+  </si>
+  <si>
+    <t>audio/s16_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s21_pq</t>
+  </si>
+  <si>
+    <t>saya nak update alamat kat identity card</t>
+  </si>
+  <si>
+    <t>audio/s21_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s22_pq</t>
+  </si>
+  <si>
+    <t>camne nak claim insurance kalau accident kereta</t>
+  </si>
+  <si>
+    <t>audio/s22_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s23_pq</t>
+  </si>
+  <si>
+    <t>nak tahu requirement untuk apply credit card</t>
+  </si>
+  <si>
+    <t>audio/s23_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s24_pq</t>
+  </si>
+  <si>
+    <t>tolong terangkan macam mana interest rate affect loan</t>
+  </si>
+  <si>
+    <t>audio/s24_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s29_pq</t>
+  </si>
+  <si>
+    <t>so how ah nak buat macam mana ni</t>
+  </si>
+  <si>
+    <t>audio/s29_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s30_pq</t>
+  </si>
+  <si>
+    <t>alamak terlupa pulak kan boleh tolong tak</t>
+  </si>
+  <si>
+    <t>audio/s30_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s31_pq</t>
+  </si>
+  <si>
+    <t>ish lambat betul lah service ni</t>
+  </si>
+  <si>
+    <t>audio/s31_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s32_pq</t>
+  </si>
+  <si>
+    <t>okay lah fine saya try dulu kot</t>
+  </si>
+  <si>
+    <t>audio/s32_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s37_pq</t>
+  </si>
+  <si>
+    <t>interest rate dia three point five percent setahun je</t>
+  </si>
+  <si>
+    <t>audio/s37_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s38_pq</t>
+  </si>
+  <si>
+    <t>kena bayar deposit dua ribu lima ratus ringgit</t>
+  </si>
+  <si>
+    <t>audio/s38_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s39_pq</t>
+  </si>
+  <si>
+    <t>cukai jualan naik dari enam peratus ke lapan peratus ke</t>
+  </si>
+  <si>
+    <t>audio/s39_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s40_pq</t>
+  </si>
+  <si>
+    <t>buka pukul nine in the morning tutup pukul five in the evening kan</t>
+  </si>
+  <si>
+    <t>audio/s40_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s45_pq</t>
+  </si>
+  <si>
+    <t>nak apply MyKad baru kat JPN macam mana</t>
+  </si>
+  <si>
+    <t>audio/s45_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s46_pq</t>
+  </si>
+  <si>
+    <t>boleh bayar bil TNB guna Maybank2u tak</t>
+  </si>
+  <si>
+    <t>audio/s46_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s47_pq</t>
+  </si>
+  <si>
+    <t>Grab dengan foodpanda mana lagi murah ah</t>
+  </si>
+  <si>
+    <t>audio/s47_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s48_pq</t>
+  </si>
+  <si>
+    <t>nak tanya pasal bantuan STR tahun ni</t>
+  </si>
+  <si>
+    <t>audio/s48_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>Phase 2 — reserve</t>
+  </si>
+  <si>
+    <t>Record only if a category comes out close, or for paired speaker analysis.</t>
+  </si>
+  <si>
+    <t>s01_pq</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>audio/s01_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s02_pq</t>
+  </si>
+  <si>
+    <t>audio/s02_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s03_pq</t>
+  </si>
+  <si>
+    <t>audio/s03_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s04_pq</t>
+  </si>
+  <si>
+    <t>audio/s04_ms_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s05_yv</t>
+  </si>
+  <si>
+    <t>audio/s05_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s06_yv</t>
+  </si>
+  <si>
+    <t>audio/s06_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s07_yv</t>
+  </si>
+  <si>
+    <t>audio/s07_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s08_yv</t>
+  </si>
+  <si>
+    <t>audio/s08_ms_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s09_pq</t>
+  </si>
+  <si>
+    <t>audio/s09_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s10_pq</t>
+  </si>
+  <si>
+    <t>audio/s10_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s11_pq</t>
+  </si>
+  <si>
+    <t>audio/s11_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s12_pq</t>
+  </si>
+  <si>
+    <t>audio/s12_en_dom_pq.wav</t>
+  </si>
+  <si>
+    <t>s13_yv</t>
+  </si>
+  <si>
+    <t>audio/s13_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s14_yv</t>
+  </si>
+  <si>
+    <t>audio/s14_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s15_yv</t>
+  </si>
+  <si>
+    <t>audio/s15_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s16_yv</t>
+  </si>
+  <si>
+    <t>audio/s16_en_dom_yv.wav</t>
+  </si>
+  <si>
+    <t>s17_pq</t>
+  </si>
+  <si>
+    <t>audio/s17_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s18_pq</t>
+  </si>
+  <si>
+    <t>audio/s18_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s19_pq</t>
+  </si>
+  <si>
+    <t>audio/s19_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s20_pq</t>
+  </si>
+  <si>
+    <t>audio/s20_balanced_pq.wav</t>
+  </si>
+  <si>
+    <t>s21_yv</t>
+  </si>
+  <si>
+    <t>audio/s21_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s22_yv</t>
+  </si>
+  <si>
+    <t>audio/s22_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s23_yv</t>
+  </si>
+  <si>
+    <t>audio/s23_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s24_yv</t>
+  </si>
+  <si>
+    <t>audio/s24_balanced_yv.wav</t>
+  </si>
+  <si>
+    <t>s25_pq</t>
+  </si>
+  <si>
+    <t>audio/s25_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s26_pq</t>
+  </si>
+  <si>
+    <t>audio/s26_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s27_pq</t>
+  </si>
+  <si>
+    <t>audio/s27_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s28_pq</t>
+  </si>
+  <si>
+    <t>audio/s28_particles_pq.wav</t>
+  </si>
+  <si>
+    <t>s29_yv</t>
+  </si>
+  <si>
+    <t>audio/s29_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s30_yv</t>
+  </si>
+  <si>
+    <t>audio/s30_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s31_yv</t>
+  </si>
+  <si>
+    <t>audio/s31_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s32_yv</t>
+  </si>
+  <si>
+    <t>audio/s32_particles_yv.wav</t>
+  </si>
+  <si>
+    <t>s33_pq</t>
+  </si>
+  <si>
+    <t>audio/s33_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s34_pq</t>
+  </si>
+  <si>
+    <t>audio/s34_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s35_pq</t>
+  </si>
+  <si>
+    <t>audio/s35_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s36_pq</t>
+  </si>
+  <si>
+    <t>audio/s36_numeric_pq.wav</t>
+  </si>
+  <si>
+    <t>s37_yv</t>
+  </si>
+  <si>
+    <t>audio/s37_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s38_yv</t>
+  </si>
+  <si>
+    <t>audio/s38_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s39_yv</t>
+  </si>
+  <si>
+    <t>audio/s39_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s40_yv</t>
+  </si>
+  <si>
+    <t>audio/s40_numeric_yv.wav</t>
+  </si>
+  <si>
+    <t>s41_pq</t>
+  </si>
+  <si>
+    <t>audio/s41_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s42_pq</t>
+  </si>
+  <si>
+    <t>audio/s42_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s43_pq</t>
+  </si>
+  <si>
+    <t>audio/s43_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s44_pq</t>
+  </si>
+  <si>
+    <t>audio/s44_entity_pq.wav</t>
+  </si>
+  <si>
+    <t>s45_yv</t>
+  </si>
+  <si>
+    <t>audio/s45_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>s46_yv</t>
+  </si>
+  <si>
+    <t>audio/s46_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>s47_yv</t>
+  </si>
+  <si>
+    <t>audio/s47_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>s48_yv</t>
+  </si>
+  <si>
+    <t>audio/s48_entity_yv.wav</t>
+  </si>
+  <si>
+    <t>yes</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="General"/>
-  </numFmts>
-  <fonts count="12">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -919,78 +933,55 @@
       <charset val="1"/>
     </font>
     <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <sz val="10"/>
-      <name val="Arial"/>
-      <family val="0"/>
-    </font>
-    <font>
-      <b val="true"/>
+      <b/>
       <sz val="13"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <color rgb="FF595959"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <i val="true"/>
+      <i/>
       <sz val="9"/>
       <color rgb="FFC00000"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FFFFFFFF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
       <sz val="10"/>
       <color rgb="FF0000FF"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
     <font>
-      <b val="true"/>
+      <b/>
       <sz val="10"/>
       <color rgb="FF1F3864"/>
       <name val="Arial"/>
-      <family val="0"/>
       <charset val="1"/>
     </font>
   </fonts>
@@ -1015,14 +1006,14 @@
     </fill>
   </fills>
   <borders count="2">
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
       <diagonal/>
     </border>
-    <border diagonalUp="false" diagonalDown="false">
+    <border>
       <left style="thin">
         <color rgb="FFD9D9D9"/>
       </left>
@@ -1038,134 +1029,41 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="20">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="43" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="41" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
-    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
+  <cellStyleXfs count="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="13">
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
+    <xf numFmtId="0" fontId="7" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="10" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="6">
+  <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Comma" xfId="15" builtinId="3"/>
-    <cellStyle name="Comma [0]" xfId="16" builtinId="6"/>
-    <cellStyle name="Currency" xfId="17" builtinId="4"/>
-    <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
-    <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="5">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF1F3864"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFFFF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FFFFFF00"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor rgb="FF0000FF"/>
-          <bgColor rgb="FF000000"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <indexedColors>
       <rgbColor rgb="FF000000"/>
@@ -1224,25 +1122,29 @@
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FF333399"/>
       <rgbColor rgb="FF333333"/>
+      <rgbColor rgb="00003366"/>
+      <rgbColor rgb="00339966"/>
+      <rgbColor rgb="00003300"/>
+      <rgbColor rgb="00333300"/>
+      <rgbColor rgb="00993300"/>
+      <rgbColor rgb="00993366"/>
+      <rgbColor rgb="00333399"/>
+      <rgbColor rgb="00333333"/>
     </indexedColors>
   </colors>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
-<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
   <a:themeElements>
     <a:clrScheme name="Office">
       <a:dk1>
@@ -1284,12 +1186,12 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Cambria" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:majorFont>
       <a:minorFont>
-        <a:latin typeface="Calibri" pitchFamily="0" charset="1"/>
+        <a:latin typeface="Calibri"/>
         <a:ea typeface=""/>
         <a:cs typeface=""/>
       </a:minorFont>
@@ -1318,7 +1220,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="1"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1339,7 +1241,7 @@
             </a:gs>
           </a:gsLst>
           <a:lin ang="16200000" scaled="0"/>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:fillStyleLst>
       <a:lnStyleLst>
@@ -1390,7 +1292,7 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
         <a:gradFill>
           <a:gsLst>
@@ -1408,36 +1310,35 @@
           <a:path path="circle">
             <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
           </a:path>
-          <a:tileRect l="0" t="0" r="0" b="0"/>
+          <a:tileRect/>
         </a:gradFill>
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:B25"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="14"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="95"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="95" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:2" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2"/>
       <c r="B2" s="2"/>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>1</v>
       </c>
@@ -1445,29 +1346,29 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A4" s="2"/>
       <c r="B4" s="2" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
       <c r="B5" s="2" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="2"/>
       <c r="B6" s="2" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="2"/>
       <c r="B7" s="2"/>
     </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="3" t="s">
         <v>6</v>
       </c>
@@ -1475,17 +1376,17 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="2"/>
       <c r="B9" s="2" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2"/>
       <c r="B10" s="2"/>
     </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>9</v>
       </c>
@@ -1493,17 +1394,17 @@
         <v>10</v>
       </c>
     </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2"/>
       <c r="B12" s="2" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="2"/>
       <c r="B13" s="2"/>
     </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="3" t="s">
         <v>12</v>
       </c>
@@ -1511,7 +1412,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
         <v>14</v>
       </c>
@@ -1519,7 +1420,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="3" t="s">
         <v>16</v>
       </c>
@@ -1527,7 +1428,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
         <v>18</v>
       </c>
@@ -1535,7 +1436,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="3" t="s">
         <v>20</v>
       </c>
@@ -1543,7 +1444,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
         <v>22</v>
       </c>
@@ -1551,7 +1452,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
@@ -1559,11 +1460,11 @@
         <v>25</v>
       </c>
     </row>
-    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="2"/>
       <c r="B21" s="2"/>
     </row>
-    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="3" t="s">
         <v>26</v>
       </c>
@@ -1571,17 +1472,17 @@
         <v>27</v>
       </c>
     </row>
-    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="2"/>
       <c r="B23" s="2" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="2"/>
       <c r="B24" s="2"/>
     </row>
-    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="3" t="s">
         <v>29</v>
       </c>
@@ -1590,55 +1491,47 @@
       </c>
     </row>
   </sheetData>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="62" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>31</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>35</v>
       </c>
@@ -1664,7 +1557,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>43</v>
       </c>
@@ -1681,10 +1574,12 @@
       <c r="F7" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="G7" s="10"/>
+      <c r="G7" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>47</v>
       </c>
@@ -1701,10 +1596,12 @@
       <c r="F8" s="9" t="s">
         <v>49</v>
       </c>
-      <c r="G8" s="10"/>
+      <c r="G8" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H8" s="11"/>
     </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>50</v>
       </c>
@@ -1721,10 +1618,12 @@
       <c r="F9" s="9" t="s">
         <v>52</v>
       </c>
-      <c r="G9" s="10"/>
+      <c r="G9" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H9" s="11"/>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>53</v>
       </c>
@@ -1741,10 +1640,12 @@
       <c r="F10" s="9" t="s">
         <v>55</v>
       </c>
-      <c r="G10" s="10"/>
+      <c r="G10" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H10" s="11"/>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>56</v>
       </c>
@@ -1761,10 +1662,12 @@
       <c r="F11" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="G11" s="10"/>
+      <c r="G11" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H11" s="11"/>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>59</v>
       </c>
@@ -1781,10 +1684,12 @@
       <c r="F12" s="9" t="s">
         <v>61</v>
       </c>
-      <c r="G12" s="10"/>
+      <c r="G12" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H12" s="11"/>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>62</v>
       </c>
@@ -1801,10 +1706,12 @@
       <c r="F13" s="9" t="s">
         <v>64</v>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H13" s="11"/>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>65</v>
       </c>
@@ -1821,10 +1728,12 @@
       <c r="F14" s="9" t="s">
         <v>67</v>
       </c>
-      <c r="G14" s="10"/>
+      <c r="G14" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H14" s="11"/>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>68</v>
       </c>
@@ -1841,10 +1750,12 @@
       <c r="F15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="G15" s="10"/>
+      <c r="G15" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H15" s="11"/>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>71</v>
       </c>
@@ -1861,10 +1772,12 @@
       <c r="F16" s="9" t="s">
         <v>73</v>
       </c>
-      <c r="G16" s="10"/>
+      <c r="G16" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H16" s="11"/>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>74</v>
       </c>
@@ -1881,10 +1794,12 @@
       <c r="F17" s="9" t="s">
         <v>76</v>
       </c>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H17" s="11"/>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>77</v>
       </c>
@@ -1901,10 +1816,12 @@
       <c r="F18" s="9" t="s">
         <v>79</v>
       </c>
-      <c r="G18" s="10"/>
+      <c r="G18" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H18" s="11"/>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>80</v>
       </c>
@@ -1921,10 +1838,12 @@
       <c r="F19" s="9" t="s">
         <v>82</v>
       </c>
-      <c r="G19" s="10"/>
+      <c r="G19" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H19" s="11"/>
     </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>83</v>
       </c>
@@ -1941,10 +1860,12 @@
       <c r="F20" s="9" t="s">
         <v>85</v>
       </c>
-      <c r="G20" s="10"/>
+      <c r="G20" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H20" s="11"/>
     </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>86</v>
       </c>
@@ -1961,10 +1882,12 @@
       <c r="F21" s="9" t="s">
         <v>88</v>
       </c>
-      <c r="G21" s="10"/>
+      <c r="G21" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H21" s="11"/>
     </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>89</v>
       </c>
@@ -1981,10 +1904,12 @@
       <c r="F22" s="9" t="s">
         <v>91</v>
       </c>
-      <c r="G22" s="10"/>
+      <c r="G22" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H22" s="11"/>
     </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:8" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>92</v>
       </c>
@@ -2003,10 +1928,12 @@
       <c r="F23" s="9" t="s">
         <v>95</v>
       </c>
-      <c r="G23" s="10"/>
+      <c r="G23" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H23" s="11"/>
     </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>96</v>
       </c>
@@ -2025,10 +1952,12 @@
       <c r="F24" s="9" t="s">
         <v>98</v>
       </c>
-      <c r="G24" s="10"/>
+      <c r="G24" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H24" s="11"/>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>99</v>
       </c>
@@ -2047,10 +1976,12 @@
       <c r="F25" s="9" t="s">
         <v>102</v>
       </c>
-      <c r="G25" s="10"/>
+      <c r="G25" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H25" s="11"/>
     </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>103</v>
       </c>
@@ -2069,10 +2000,12 @@
       <c r="F26" s="9" t="s">
         <v>105</v>
       </c>
-      <c r="G26" s="10"/>
+      <c r="G26" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H26" s="11"/>
     </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>106</v>
       </c>
@@ -2089,10 +2022,12 @@
       <c r="F27" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H27" s="11"/>
     </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>109</v>
       </c>
@@ -2109,10 +2044,12 @@
       <c r="F28" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="G28" s="10"/>
+      <c r="G28" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H28" s="11"/>
     </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>112</v>
       </c>
@@ -2129,10 +2066,12 @@
       <c r="F29" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="G29" s="10"/>
+      <c r="G29" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H29" s="11"/>
     </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>115</v>
       </c>
@@ -2149,76 +2088,69 @@
       <c r="F30" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="G30" s="10"/>
+      <c r="G30" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H30" s="11"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B32" s="12" t="str">
-        <f aca="false">COUNTIF(G7:G30,"yes")&amp;" of "&amp;24&amp;"  ("&amp;TEXT(COUNTIF(G7:G30,"yes")/24,"0%")&amp;" done)"</f>
-        <v>0 of 24  (0% done)</v>
+        <f>COUNTIF(G7:G30,"yes")&amp;" of "&amp;24&amp;"  ("&amp;TEXT(COUNTIF(G7:G30,"yes")/24,"0%")&amp;" done)"</f>
+        <v>24 of 24  (100% done)</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H30"/>
+  <autoFilter ref="A6:H30" xr:uid="{00000000-0009-0000-0000-000001000000}"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G7:G30" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="G7:G30" xr:uid="{00000000-0002-0000-0100-000000000000}">
       <formula1>"no,yes"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:H32"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="62" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>35</v>
       </c>
@@ -2244,7 +2176,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>120</v>
       </c>
@@ -2261,10 +2193,12 @@
       <c r="F7" s="9" t="s">
         <v>122</v>
       </c>
-      <c r="G7" s="10"/>
+      <c r="G7" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>123</v>
       </c>
@@ -2281,10 +2215,12 @@
       <c r="F8" s="9" t="s">
         <v>125</v>
       </c>
-      <c r="G8" s="10"/>
+      <c r="G8" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H8" s="11"/>
     </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>126</v>
       </c>
@@ -2301,10 +2237,12 @@
       <c r="F9" s="9" t="s">
         <v>128</v>
       </c>
-      <c r="G9" s="10"/>
+      <c r="G9" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H9" s="11"/>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>129</v>
       </c>
@@ -2321,10 +2259,12 @@
       <c r="F10" s="9" t="s">
         <v>131</v>
       </c>
-      <c r="G10" s="10"/>
+      <c r="G10" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H10" s="11"/>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>132</v>
       </c>
@@ -2341,10 +2281,12 @@
       <c r="F11" s="9" t="s">
         <v>134</v>
       </c>
-      <c r="G11" s="10"/>
+      <c r="G11" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H11" s="11"/>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>135</v>
       </c>
@@ -2361,10 +2303,12 @@
       <c r="F12" s="9" t="s">
         <v>137</v>
       </c>
-      <c r="G12" s="10"/>
+      <c r="G12" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H12" s="11"/>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>138</v>
       </c>
@@ -2381,10 +2325,12 @@
       <c r="F13" s="9" t="s">
         <v>140</v>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H13" s="11"/>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>141</v>
       </c>
@@ -2401,10 +2347,12 @@
       <c r="F14" s="9" t="s">
         <v>143</v>
       </c>
-      <c r="G14" s="10"/>
+      <c r="G14" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H14" s="11"/>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>144</v>
       </c>
@@ -2421,10 +2369,12 @@
       <c r="F15" s="9" t="s">
         <v>146</v>
       </c>
-      <c r="G15" s="10"/>
+      <c r="G15" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H15" s="11"/>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>147</v>
       </c>
@@ -2441,10 +2391,12 @@
       <c r="F16" s="9" t="s">
         <v>149</v>
       </c>
-      <c r="G16" s="10"/>
+      <c r="G16" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H16" s="11"/>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>150</v>
       </c>
@@ -2461,10 +2413,12 @@
       <c r="F17" s="9" t="s">
         <v>152</v>
       </c>
-      <c r="G17" s="10"/>
+      <c r="G17" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H17" s="11"/>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>153</v>
       </c>
@@ -2481,10 +2435,12 @@
       <c r="F18" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="G18" s="10"/>
+      <c r="G18" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H18" s="11"/>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>156</v>
       </c>
@@ -2501,10 +2457,12 @@
       <c r="F19" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="G19" s="10"/>
+      <c r="G19" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H19" s="11"/>
     </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>159</v>
       </c>
@@ -2521,10 +2479,12 @@
       <c r="F20" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="G20" s="10"/>
+      <c r="G20" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H20" s="11"/>
     </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>162</v>
       </c>
@@ -2541,10 +2501,12 @@
       <c r="F21" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="G21" s="10"/>
+      <c r="G21" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H21" s="11"/>
     </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>165</v>
       </c>
@@ -2561,10 +2523,12 @@
       <c r="F22" s="9" t="s">
         <v>167</v>
       </c>
-      <c r="G22" s="10"/>
+      <c r="G22" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H22" s="11"/>
     </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>168</v>
       </c>
@@ -2583,10 +2547,12 @@
       <c r="F23" s="9" t="s">
         <v>170</v>
       </c>
-      <c r="G23" s="10"/>
+      <c r="G23" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H23" s="11"/>
     </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>171</v>
       </c>
@@ -2605,10 +2571,12 @@
       <c r="F24" s="9" t="s">
         <v>173</v>
       </c>
-      <c r="G24" s="10"/>
+      <c r="G24" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H24" s="11"/>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>174</v>
       </c>
@@ -2627,10 +2595,12 @@
       <c r="F25" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="G25" s="10"/>
+      <c r="G25" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H25" s="11"/>
     </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>177</v>
       </c>
@@ -2649,10 +2619,12 @@
       <c r="F26" s="9" t="s">
         <v>179</v>
       </c>
-      <c r="G26" s="10"/>
+      <c r="G26" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H26" s="11"/>
     </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>180</v>
       </c>
@@ -2669,10 +2641,12 @@
       <c r="F27" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="G27" s="10"/>
+      <c r="G27" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H27" s="11"/>
     </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>183</v>
       </c>
@@ -2689,10 +2663,12 @@
       <c r="F28" s="9" t="s">
         <v>185</v>
       </c>
-      <c r="G28" s="10"/>
+      <c r="G28" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H28" s="11"/>
     </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>186</v>
       </c>
@@ -2709,10 +2685,12 @@
       <c r="F29" s="9" t="s">
         <v>188</v>
       </c>
-      <c r="G29" s="10"/>
+      <c r="G29" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H29" s="11"/>
     </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>189</v>
       </c>
@@ -2729,76 +2707,69 @@
       <c r="F30" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="G30" s="10"/>
+      <c r="G30" s="10" t="s">
+        <v>291</v>
+      </c>
       <c r="H30" s="11"/>
     </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B32" s="12" t="str">
-        <f aca="false">COUNTIF(G7:G30,"yes")&amp;" of "&amp;24&amp;"  ("&amp;TEXT(COUNTIF(G7:G30,"yes")/24,"0%")&amp;" done)"</f>
-        <v>0 of 24  (0% done)</v>
+        <f>COUNTIF(G7:G30,"yes")&amp;" of "&amp;24&amp;"  ("&amp;TEXT(COUNTIF(G7:G30,"yes")/24,"0%")&amp;" done)"</f>
+        <v>24 of 24  (100% done)</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H30"/>
+  <autoFilter ref="A6:H30" xr:uid="{00000000-0009-0000-0000-000002000000}"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G7:G30" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="G7:G30" xr:uid="{00000000-0002-0000-0200-000000000000}">
       <formula1>"no,yes"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <sheetPr filterMode="false">
-    <pageSetUpPr fitToPage="false"/>
-  </sheetPr>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H56"/>
-  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="false" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="62"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="16"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="32"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="0" width="11"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="0" width="24"/>
+    <col min="1" max="1" width="12" customWidth="1"/>
+    <col min="2" max="2" width="62" customWidth="1"/>
+    <col min="3" max="3" width="12" customWidth="1"/>
+    <col min="4" max="4" width="16" customWidth="1"/>
+    <col min="5" max="5" width="7" customWidth="1"/>
+    <col min="6" max="6" width="32" customWidth="1"/>
+    <col min="7" max="7" width="11" customWidth="1"/>
+    <col min="8" max="8" width="24" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="16.15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="1" spans="1:8" ht="16.5" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>192</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="4" t="s">
         <v>193</v>
       </c>
     </row>
-    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="4" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>35</v>
       </c>
@@ -2824,7 +2795,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="7" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>194</v>
       </c>
@@ -2844,7 +2815,7 @@
       <c r="G7" s="10"/>
       <c r="H7" s="11"/>
     </row>
-    <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="8" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>197</v>
       </c>
@@ -2864,7 +2835,7 @@
       <c r="G8" s="10"/>
       <c r="H8" s="11"/>
     </row>
-    <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="9" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="7" t="s">
         <v>199</v>
       </c>
@@ -2884,7 +2855,7 @@
       <c r="G9" s="10"/>
       <c r="H9" s="11"/>
     </row>
-    <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="10" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7" t="s">
         <v>201</v>
       </c>
@@ -2904,7 +2875,7 @@
       <c r="G10" s="10"/>
       <c r="H10" s="11"/>
     </row>
-    <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="11" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="7" t="s">
         <v>203</v>
       </c>
@@ -2924,7 +2895,7 @@
       <c r="G11" s="10"/>
       <c r="H11" s="11"/>
     </row>
-    <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="12" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="7" t="s">
         <v>205</v>
       </c>
@@ -2944,7 +2915,7 @@
       <c r="G12" s="10"/>
       <c r="H12" s="11"/>
     </row>
-    <row r="13" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="13" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>207</v>
       </c>
@@ -2964,7 +2935,7 @@
       <c r="G13" s="10"/>
       <c r="H13" s="11"/>
     </row>
-    <row r="14" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="14" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="7" t="s">
         <v>209</v>
       </c>
@@ -2984,7 +2955,7 @@
       <c r="G14" s="10"/>
       <c r="H14" s="11"/>
     </row>
-    <row r="15" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="15" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>211</v>
       </c>
@@ -3004,7 +2975,7 @@
       <c r="G15" s="10"/>
       <c r="H15" s="11"/>
     </row>
-    <row r="16" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="16" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>213</v>
       </c>
@@ -3024,7 +2995,7 @@
       <c r="G16" s="10"/>
       <c r="H16" s="11"/>
     </row>
-    <row r="17" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="17" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="7" t="s">
         <v>215</v>
       </c>
@@ -3044,7 +3015,7 @@
       <c r="G17" s="10"/>
       <c r="H17" s="11"/>
     </row>
-    <row r="18" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="18" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="7" t="s">
         <v>217</v>
       </c>
@@ -3064,7 +3035,7 @@
       <c r="G18" s="10"/>
       <c r="H18" s="11"/>
     </row>
-    <row r="19" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="19" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>219</v>
       </c>
@@ -3084,7 +3055,7 @@
       <c r="G19" s="10"/>
       <c r="H19" s="11"/>
     </row>
-    <row r="20" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="20" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>221</v>
       </c>
@@ -3104,7 +3075,7 @@
       <c r="G20" s="10"/>
       <c r="H20" s="11"/>
     </row>
-    <row r="21" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="21" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>223</v>
       </c>
@@ -3124,7 +3095,7 @@
       <c r="G21" s="10"/>
       <c r="H21" s="11"/>
     </row>
-    <row r="22" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="22" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="7" t="s">
         <v>225</v>
       </c>
@@ -3144,7 +3115,7 @@
       <c r="G22" s="10"/>
       <c r="H22" s="11"/>
     </row>
-    <row r="23" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="23" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="7" t="s">
         <v>227</v>
       </c>
@@ -3164,7 +3135,7 @@
       <c r="G23" s="10"/>
       <c r="H23" s="11"/>
     </row>
-    <row r="24" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="24" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="7" t="s">
         <v>229</v>
       </c>
@@ -3184,7 +3155,7 @@
       <c r="G24" s="10"/>
       <c r="H24" s="11"/>
     </row>
-    <row r="25" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="25" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>231</v>
       </c>
@@ -3204,7 +3175,7 @@
       <c r="G25" s="10"/>
       <c r="H25" s="11"/>
     </row>
-    <row r="26" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="26" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="7" t="s">
         <v>233</v>
       </c>
@@ -3224,7 +3195,7 @@
       <c r="G26" s="10"/>
       <c r="H26" s="11"/>
     </row>
-    <row r="27" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="27" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
         <v>235</v>
       </c>
@@ -3244,7 +3215,7 @@
       <c r="G27" s="10"/>
       <c r="H27" s="11"/>
     </row>
-    <row r="28" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="28" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="7" t="s">
         <v>237</v>
       </c>
@@ -3264,7 +3235,7 @@
       <c r="G28" s="10"/>
       <c r="H28" s="11"/>
     </row>
-    <row r="29" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="29" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>239</v>
       </c>
@@ -3284,7 +3255,7 @@
       <c r="G29" s="10"/>
       <c r="H29" s="11"/>
     </row>
-    <row r="30" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="30" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>241</v>
       </c>
@@ -3304,7 +3275,7 @@
       <c r="G30" s="10"/>
       <c r="H30" s="11"/>
     </row>
-    <row r="31" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="31" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>243</v>
       </c>
@@ -3324,7 +3295,7 @@
       <c r="G31" s="10"/>
       <c r="H31" s="11"/>
     </row>
-    <row r="32" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="32" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="7" t="s">
         <v>245</v>
       </c>
@@ -3344,7 +3315,7 @@
       <c r="G32" s="10"/>
       <c r="H32" s="11"/>
     </row>
-    <row r="33" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="33" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
         <v>247</v>
       </c>
@@ -3364,7 +3335,7 @@
       <c r="G33" s="10"/>
       <c r="H33" s="11"/>
     </row>
-    <row r="34" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="34" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>249</v>
       </c>
@@ -3384,7 +3355,7 @@
       <c r="G34" s="10"/>
       <c r="H34" s="11"/>
     </row>
-    <row r="35" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="35" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
         <v>251</v>
       </c>
@@ -3404,7 +3375,7 @@
       <c r="G35" s="10"/>
       <c r="H35" s="11"/>
     </row>
-    <row r="36" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="36" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>253</v>
       </c>
@@ -3424,7 +3395,7 @@
       <c r="G36" s="10"/>
       <c r="H36" s="11"/>
     </row>
-    <row r="37" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="37" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>255</v>
       </c>
@@ -3444,7 +3415,7 @@
       <c r="G37" s="10"/>
       <c r="H37" s="11"/>
     </row>
-    <row r="38" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="38" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="7" t="s">
         <v>257</v>
       </c>
@@ -3464,7 +3435,7 @@
       <c r="G38" s="10"/>
       <c r="H38" s="11"/>
     </row>
-    <row r="39" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="39" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>259</v>
       </c>
@@ -3486,7 +3457,7 @@
       <c r="G39" s="10"/>
       <c r="H39" s="11"/>
     </row>
-    <row r="40" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="40" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="7" t="s">
         <v>261</v>
       </c>
@@ -3508,7 +3479,7 @@
       <c r="G40" s="10"/>
       <c r="H40" s="11"/>
     </row>
-    <row r="41" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="41" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
         <v>263</v>
       </c>
@@ -3530,7 +3501,7 @@
       <c r="G41" s="10"/>
       <c r="H41" s="11"/>
     </row>
-    <row r="42" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="42" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="7" t="s">
         <v>265</v>
       </c>
@@ -3552,7 +3523,7 @@
       <c r="G42" s="10"/>
       <c r="H42" s="11"/>
     </row>
-    <row r="43" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="43" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
         <v>267</v>
       </c>
@@ -3574,7 +3545,7 @@
       <c r="G43" s="10"/>
       <c r="H43" s="11"/>
     </row>
-    <row r="44" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="44" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>269</v>
       </c>
@@ -3596,7 +3567,7 @@
       <c r="G44" s="10"/>
       <c r="H44" s="11"/>
     </row>
-    <row r="45" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="45" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>271</v>
       </c>
@@ -3618,7 +3589,7 @@
       <c r="G45" s="10"/>
       <c r="H45" s="11"/>
     </row>
-    <row r="46" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="46" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="7" t="s">
         <v>273</v>
       </c>
@@ -3640,7 +3611,7 @@
       <c r="G46" s="10"/>
       <c r="H46" s="11"/>
     </row>
-    <row r="47" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="47" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>275</v>
       </c>
@@ -3660,7 +3631,7 @@
       <c r="G47" s="10"/>
       <c r="H47" s="11"/>
     </row>
-    <row r="48" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="48" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="7" t="s">
         <v>277</v>
       </c>
@@ -3680,7 +3651,7 @@
       <c r="G48" s="10"/>
       <c r="H48" s="11"/>
     </row>
-    <row r="49" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="49" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
         <v>279</v>
       </c>
@@ -3700,7 +3671,7 @@
       <c r="G49" s="10"/>
       <c r="H49" s="11"/>
     </row>
-    <row r="50" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="50" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>281</v>
       </c>
@@ -3720,7 +3691,7 @@
       <c r="G50" s="10"/>
       <c r="H50" s="11"/>
     </row>
-    <row r="51" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="51" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
         <v>283</v>
       </c>
@@ -3740,7 +3711,7 @@
       <c r="G51" s="10"/>
       <c r="H51" s="11"/>
     </row>
-    <row r="52" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="52" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="7" t="s">
         <v>285</v>
       </c>
@@ -3760,7 +3731,7 @@
       <c r="G52" s="10"/>
       <c r="H52" s="11"/>
     </row>
-    <row r="53" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="53" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
         <v>287</v>
       </c>
@@ -3780,7 +3751,7 @@
       <c r="G53" s="10"/>
       <c r="H53" s="11"/>
     </row>
-    <row r="54" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="54" spans="1:8" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="7" t="s">
         <v>289</v>
       </c>
@@ -3800,30 +3771,24 @@
       <c r="G54" s="10"/>
       <c r="H54" s="11"/>
     </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56" s="3" t="s">
         <v>118</v>
       </c>
       <c r="B56" s="12" t="str">
-        <f aca="false">COUNTIF(G7:G54,"yes")&amp;" of "&amp;48&amp;"  ("&amp;TEXT(COUNTIF(G7:G54,"yes")/48,"0%")&amp;" done)"</f>
+        <f>COUNTIF(G7:G54,"yes")&amp;" of "&amp;48&amp;"  ("&amp;TEXT(COUNTIF(G7:G54,"yes")/48,"0%")&amp;" done)"</f>
         <v>0 of 48  (0% done)</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A6:H54"/>
+  <autoFilter ref="A6:H54" xr:uid="{00000000-0009-0000-0000-000003000000}"/>
   <dataValidations count="1">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="false" showInputMessage="false" sqref="G7:G54" type="list">
+    <dataValidation type="list" allowBlank="1" sqref="G7:G54" xr:uid="{00000000-0002-0000-0300-000000000000}">
       <formula1>"no,yes"</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
-  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
-  <headerFooter differentFirst="false" differentOddEven="false">
-    <oddHeader/>
-    <oddFooter/>
-  </headerFooter>
-  <drawing r:id="rId1"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
 </worksheet>
 </file>
</xml_diff>